<commit_message>
Add: cara buka chrome via python
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi Mei 02 2026 Saturday 08_54_42.xlsx
+++ b/PC-06/docs/Absensi Mei 02 2026 Saturday 08_54_42.xlsx
@@ -1285,7 +1285,11 @@
       <c r="D10" s="12" t="n"/>
       <c r="E10" s="12" t="n"/>
       <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H10" s="12" t="n"/>
       <c r="I10" s="12" t="n"/>
       <c r="J10" s="12" t="n"/>
@@ -1340,7 +1344,11 @@
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
       <c r="J11" s="8" t="n"/>
@@ -1390,7 +1398,11 @@
       <c r="D12" s="8" t="n"/>
       <c r="E12" s="8" t="n"/>
       <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
       <c r="J12" s="8" t="n"/>
@@ -5862,7 +5874,11 @@
         </is>
       </c>
       <c r="D35" s="8" t="n"/>
-      <c r="E35" s="8" t="n"/>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
       <c r="H35" s="8" t="n"/>
@@ -11558,7 +11574,11 @@
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n"/>
@@ -12375,7 +12395,11 @@
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="n"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>

</xml_diff>

<commit_message>
Absensi Mei 2026 - update TKB1, TKa, TKB2, PG
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi Mei 02 2026 Saturday 08_54_42.xlsx
+++ b/PC-06/docs/Absensi Mei 02 2026 Saturday 08_54_42.xlsx
@@ -7515,7 +7515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO55"/>
+  <dimension ref="A1:AW55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -9658,7 +9658,11 @@
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
-      <c r="H42" s="8" t="n"/>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="I42" s="8" t="n"/>
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>

</xml_diff>